<commit_message>
Add Excel-driven member workflow and site updates
Switch site to use contents/member-info.xlsx as the single source of truth for member data and update the build pipeline and docs accordingly. Updates include: adding .gitignore/.claudeignore and new image assets; documenting excel_to_content.py in README/STRUCTURE/CLAUDE and requiring openpyxl; adding templates/partials/subpage-header.html; updating build.py to load per-member JSON (members_by_id) and to recursively walk articles (preserve nested paths); many per-member position text tweaks and small member JSON name casing fixes; add new group-life image and generated WebP assets; remove create_member_excel.py and delete several legacy export/member extract files; update CONTRIBUTING to instruct editing the spreadsheet rather than hand-editing members.json. These changes enable auto-generation of members.json, per-member JSON/Markdown, and streamline builds to derive pages from the spreadsheet.
</commit_message>
<xml_diff>
--- a/contents/member-info.xlsx
+++ b/contents/member-info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/Github/NTU-E3-Center.github.io/contents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39FC56E-CBE6-D34E-A05E-D5F8410AF0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79114A5-CC33-5441-972A-FC31918539D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="244">
   <si>
     <t>WebID</t>
   </si>
@@ -265,11 +264,6 @@
     <t>Harper completed her **B.S. in Civil Engineering** at National Central University (NCU), Taoyuan, in 2023, and pursued her graduate studies in the Computer-Aided Engineering (CAE) division of the Civil Engineering Department at National Taiwan University (NTU). In February 2025, she advanced directly into the **Ph.D. program** at NTU. Her research focuses on computer vision applications, with particular interests in medical imaging analysis and energy forecasting.</t>
   </si>
   <si>
-    <t>Ph.D. Student,
-Department of Civil Engineering,
-National Taiwan University</t>
-  </si>
-  <si>
     <t>/ Computer Vision 
 / Medical Image Analysis 
 / Energy Forecasting</t>
@@ -292,11 +286,6 @@
   <si>
     <t>Ray is a **Ph.D. student** at National Taiwan University, specializing in the intersection of **data analytics, artificial intelligence (AI), and Geographic Information Systems (GIS)**. His research is driven by a focus on green mobility, environmental policy, and energy economics, with a dedicated interest in leveraging data-driven decision-making to advance global net-zero goals and the development of sustainable smart cities.
 With a strong technical background in machine learning and spatial analysis, Ray focuses on modeling complex urban systems to inform more effective environmental strategies. He is committed to interdisciplinary collaboration and is actively involved in research initiatives that bridge the gap between advanced computational techniques and actionable policy frameworks.</t>
-  </si>
-  <si>
-    <t>Ph.D. Student,
-Department of Civil Engineering,
-National Taiwan University.</t>
   </si>
   <si>
     <t>/ Green Mobility &amp; Sustainable Transport 
@@ -350,11 +339,6 @@
     <t>Derek graduated from the **Department of Chemical Engineering** at National Taiwan University of Science and Technology in 2024. He is currently pursuing a **master’s degree** at the Graduate Institute of Chemical Engineering at National Taiwan University, under the guidance of Professor Lisa Hsieh. His current research focuses on **sustainable supply chains**, including topics such as **Green Vehicle Routing Problems (Green VRP)**, joint distribution, and hub-and-spoke network design.</t>
   </si>
   <si>
-    <t>Master's Student,
-Department of Chemical Engineering,
-National Taiwan University</t>
-  </si>
-  <si>
     <t>/ Sustainable Supply Chain Management 
 / Green Vehicle Routing Problems (Green VRP) 
 / Joint Distribution Systems 
@@ -394,11 +378,6 @@
     <t>Leo, also known by the nickname **DuoDuo(多多)**, completed his **undergraduate degree in Civil Engineering** at National Taiwan University (NTU) in 2025. He is currently a member of the **Computer-Aided Engineering (CAE)** division of NTU’s Civil Engineering department. His interests include playing volleyball, board games, and exploring new experiences. His research focuses on integrating **large language models (LLMs)** with **computer vision** to control autonomous vehicles, aiming to ensure safe driving, provide transparent explanations of model decisions, and optimize energy efficiency.</t>
   </si>
   <si>
-    <t>Master's Student,
-Department of Civil Engineering,
-National Taiwan University</t>
-  </si>
-  <si>
     <t>/ Autonomous Vehicles 
 / Computer Vision</t>
   </si>
@@ -481,10 +460,6 @@
   </si>
   <si>
     <t>Yi-Fang is a **graduate student** in the **Master’s Program in Disaster Risk Reduction and Resilience** at National Taiwan University, with a background in **civil engineering** and professional experience in large-scale energy infrastructure projects. Her research focuses on **energy planning**, with particular interest in integrating climate change risk assessment, resilience strategies, and sustainable energy systems. Prior to her graduate studies, she worked as a **civil engineer** and **project coordination specialist** on offshore substation construction projects, and later as a **research assistant** on climate change adaptation planning for Taiwan’s national parks. She is especially interested in bridging the fields of infrastructure development, climate resilience, and renewable energy to support sustainable transitions in both urban and natural environments.</t>
-  </si>
-  <si>
-    <t>Master’s Program in Disaster Risk Reduction and Resilience,
-National Taiwan University</t>
   </si>
   <si>
     <t>/ Sustainable Energy Planning</t>
@@ -735,76 +710,115 @@
     <t>Yu Fang Shen</t>
   </si>
   <si>
-    <t>CHIH-YA CHENG</t>
-  </si>
-  <si>
     <t>Chun-Hao Huang</t>
   </si>
   <si>
-    <t>HIGASHI MASAKI</t>
-  </si>
-  <si>
     <t>Yugo</t>
   </si>
   <si>
     <t>Masaki</t>
   </si>
   <si>
-    <t>Master's Student,
+    <t>Undergraduate (Pre-Master's) Student</t>
+  </si>
+  <si>
+    <t>An-Ching Chung</t>
+  </si>
+  <si>
+    <t>Yi-Ya Yu</t>
+  </si>
+  <si>
+    <t>Hsun-Yen Wu</t>
+  </si>
+  <si>
+    <t>Shao Yang Cheung</t>
+  </si>
+  <si>
+    <t>Yu-Ting Huang</t>
+  </si>
+  <si>
+    <t>Yu-Shin Hu</t>
+  </si>
+  <si>
+    <t>Pei-Ci Chen</t>
+  </si>
+  <si>
+    <t>Kai-Yun Lo</t>
+  </si>
+  <si>
+    <t>Yi-Fan Feng</t>
+  </si>
+  <si>
+    <t>Jing-Siou Tseng</t>
+  </si>
+  <si>
+    <t>Yuan-Shin Fu</t>
+  </si>
+  <si>
+    <t>Chia-Yu Tsai</t>
+  </si>
+  <si>
+    <t>Tsung-Heng Chang</t>
+  </si>
+  <si>
+    <t>Wei-Hsuan Chen</t>
+  </si>
+  <si>
+    <t>Yu-Jui Chang</t>
+  </si>
+  <si>
+    <t>Cheng-Ye Li</t>
+  </si>
+  <si>
+    <t>Chih-Ya Cheng</t>
+  </si>
+  <si>
+    <t>Higashi Masaki</t>
+  </si>
+  <si>
+    <t>Year 2 Ph.D. Student,
+Department of Civil Engineering,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 1 Ph.D. Student,
+Department of Civil Engineering,
+National Taiwan University.</t>
+  </si>
+  <si>
+    <t>Year 1 Master's Student,
 Department of Civil Engineering,
 National Taiwan University
 (Double Degree from Kyushu University)</t>
   </si>
   <si>
-    <t>Undergraduate (Pre-Master's) Student</t>
-  </si>
-  <si>
-    <t>An-Ching Chung</t>
-  </si>
-  <si>
-    <t>Yi-Ya Yu</t>
-  </si>
-  <si>
-    <t>Hsun-Yen Wu</t>
-  </si>
-  <si>
-    <t>Shao Yang Cheung</t>
-  </si>
-  <si>
-    <t>Yu-Ting Huang</t>
-  </si>
-  <si>
-    <t>Yu-Shin Hu</t>
-  </si>
-  <si>
-    <t>Pei-Ci Chen</t>
-  </si>
-  <si>
-    <t>Kai-Yun Lo</t>
-  </si>
-  <si>
-    <t>Yi-Fan Feng</t>
-  </si>
-  <si>
-    <t>Jing-Siou Tseng</t>
-  </si>
-  <si>
-    <t>Yuan-Shin Fu</t>
-  </si>
-  <si>
-    <t>Chia-Yu Tsai</t>
-  </si>
-  <si>
-    <t>Tsung-Heng Chang</t>
-  </si>
-  <si>
-    <t>Wei-Hsuan Chen</t>
-  </si>
-  <si>
-    <t>Yu-Jui Chang</t>
-  </si>
-  <si>
-    <t>Cheng-Ye Li</t>
+    <t>Year 3 Master's Student (Part-time),
+Department of Civil Engineering,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 2 Master's Student,
+Department of Civil Engineering,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 2 Master's Student,
+Department of Chemical Engineering,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 1 Master’s Program in Disaster Risk Reduction and Resilience,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 1 Master's Student,
+Department of Civil Engineering,
+National Taiwan University</t>
+  </si>
+  <si>
+    <t>Year 1 Master's Student,
+Department of Chemical Engineering,
+National Taiwan University</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>2</v>
@@ -1264,7 +1278,7 @@
         <v>44</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="H2" s="1" t="str">
         <f t="shared" ref="H2:H38" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(G2),"-","")," ",""))</f>
@@ -1319,7 +1333,7 @@
         <v>27</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="H3" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1374,7 +1388,7 @@
         <v>38</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="H4" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1476,13 +1490,13 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="H6" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1529,7 +1543,7 @@
         <v>59</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="H7" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1551,11 +1565,11 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1" t="s">
-        <v>69</v>
+        <v>235</v>
       </c>
       <c r="Q7" s="1"/>
       <c r="R7" s="1" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -1602,10 +1616,10 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q8" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="R8" s="1" t="s">
         <v>68</v>
@@ -1616,32 +1630,32 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="H9" s="1" t="str">
         <f t="shared" si="0"/>
         <v>hungjuilin</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>60</v>
@@ -1655,13 +1669,13 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1" t="s">
-        <v>77</v>
+        <v>236</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="112" x14ac:dyDescent="0.2">
@@ -1669,22 +1683,22 @@
         <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="H10" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1692,13 +1706,13 @@
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>67</v>
@@ -1706,7 +1720,7 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -1716,7 +1730,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>36</v>
@@ -1725,13 +1739,13 @@
         <v>57</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="H11" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1739,10 +1753,10 @@
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L11" s="1" t="s">
         <v>61</v>
@@ -1753,7 +1767,7 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1" t="s">
-        <v>107</v>
+        <v>238</v>
       </c>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
@@ -1763,22 +1777,22 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="H12" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1786,10 +1800,10 @@
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>61</v>
@@ -1800,7 +1814,7 @@
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1" t="s">
-        <v>107</v>
+        <v>239</v>
       </c>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -1810,22 +1824,22 @@
         <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="H13" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1833,10 +1847,10 @@
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>61</v>
@@ -1847,7 +1861,7 @@
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1" t="s">
-        <v>107</v>
+        <v>239</v>
       </c>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
@@ -1857,35 +1871,35 @@
         <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="H14" s="1" t="str">
         <f t="shared" si="0"/>
         <v>enyichou</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L14" s="1" t="s">
         <v>61</v>
@@ -1896,13 +1910,13 @@
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1" t="s">
-        <v>94</v>
+        <v>240</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="64" x14ac:dyDescent="0.2">
@@ -1910,38 +1924,38 @@
         <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H15" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yifangchang</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>67</v>
@@ -1949,13 +1963,13 @@
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1" t="s">
-        <v>135</v>
+        <v>241</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -1963,38 +1977,38 @@
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H16" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>shuochenli</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L16" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H16" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>shuochenli</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>67</v>
@@ -2002,13 +2016,13 @@
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1" t="s">
-        <v>107</v>
+        <v>242</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2016,38 +2030,38 @@
         <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H17" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yurankeng</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M17" s="1" t="s">
         <v>67</v>
@@ -2055,13 +2069,13 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1" t="s">
-        <v>94</v>
+        <v>243</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2069,22 +2083,22 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="H18" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2092,13 +2106,13 @@
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>67</v>
@@ -2106,7 +2120,7 @@
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1" t="s">
-        <v>107</v>
+        <v>242</v>
       </c>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
@@ -2116,38 +2130,38 @@
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="H19" s="1" t="str">
         <f t="shared" si="0"/>
         <v>houchuanchen</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>67</v>
@@ -2155,13 +2169,13 @@
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1" t="s">
-        <v>107</v>
+        <v>242</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2169,22 +2183,22 @@
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="H20" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2192,13 +2206,13 @@
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M20" s="1" t="s">
         <v>67</v>
@@ -2206,7 +2220,7 @@
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1" t="s">
-        <v>94</v>
+        <v>243</v>
       </c>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
@@ -2216,22 +2230,22 @@
         <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="H21" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2239,13 +2253,13 @@
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L21" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="M21" s="1" t="s">
         <v>67</v>
@@ -2253,7 +2267,7 @@
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
@@ -2263,22 +2277,22 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="H22" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2286,13 +2300,13 @@
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>67</v>
@@ -2300,7 +2314,7 @@
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
@@ -2310,22 +2324,22 @@
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="H23" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2333,13 +2347,13 @@
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>67</v>
@@ -2347,7 +2361,7 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
@@ -2357,22 +2371,22 @@
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="H24" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2380,13 +2394,13 @@
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>67</v>
@@ -2394,7 +2408,7 @@
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
@@ -2404,35 +2418,35 @@
         <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="E25" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="H25" s="1" t="str">
         <f t="shared" si="0"/>
         <v>chunhaohuang</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="M25" s="1" t="s">
         <v>67</v>
@@ -2440,7 +2454,7 @@
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
@@ -2450,32 +2464,32 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="H26" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yugoimoto</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>52</v>
@@ -2496,35 +2510,35 @@
         <v>24</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="H27" s="1" t="str">
         <f t="shared" si="0"/>
         <v>chiayutsai</v>
       </c>
       <c r="J27" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K27" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="L27" s="1" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>31</v>
@@ -2540,35 +2554,35 @@
         <v>25</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="H28" s="1" t="str">
         <f t="shared" si="0"/>
         <v>tsunghengchang</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>31</v>
@@ -2584,7 +2598,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>24</v>
@@ -2593,23 +2607,23 @@
         <v>57</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="H29" s="1" t="str">
         <f t="shared" si="0"/>
         <v>kaiyunlo</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L29" s="1" t="s">
         <v>30</v>
@@ -2628,32 +2642,32 @@
         <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>37</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="H30" s="1" t="str">
         <f t="shared" si="0"/>
         <v>weihsuanchen</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L30" s="1" t="s">
         <v>30</v>
@@ -2672,7 +2686,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>24</v>
@@ -2681,23 +2695,23 @@
         <v>57</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="H31" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yifanfeng</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L31" s="1" t="s">
         <v>30</v>
@@ -2716,22 +2730,22 @@
         <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>36</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="H32" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2739,10 +2753,10 @@
       </c>
       <c r="I32" s="1"/>
       <c r="J32" s="1" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>39</v>
@@ -2761,7 +2775,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>36</v>
@@ -2770,13 +2784,13 @@
         <v>57</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="H33" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2784,10 +2798,10 @@
       </c>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>39</v>
@@ -2806,7 +2820,7 @@
         <v>31</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>36</v>
@@ -2815,26 +2829,26 @@
         <v>57</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H34" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yuanhsichien</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>39</v>
@@ -2845,11 +2859,11 @@
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="Q34" s="1"/>
       <c r="R34" s="1" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
@@ -2857,22 +2871,22 @@
         <v>32</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="H35" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2880,10 +2894,10 @@
       </c>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>52</v>
@@ -2902,22 +2916,22 @@
         <v>33</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>48</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="H36" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2925,10 +2939,10 @@
       </c>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>52</v>
@@ -2947,7 +2961,7 @@
         <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>48</v>
@@ -2956,13 +2970,13 @@
         <v>57</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="H37" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2970,10 +2984,10 @@
       </c>
       <c r="I37" s="1"/>
       <c r="J37" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L37" s="1" t="s">
         <v>52</v>
@@ -2992,7 +3006,7 @@
         <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>48</v>
@@ -3001,13 +3015,13 @@
         <v>57</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="H38" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3015,10 +3029,10 @@
       </c>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Add news item and render pipeline for news pages
Publish a new news article (2026 NTU-UG Joint Seminar) with accompanying images and assets, and wire up site rendering for news item pages. Changes include: added markdown article and image assets under contents/, added pre-generated assets under docs/assets/, added a news-item template and CSS (templates/pages/news/news-item.html, docs/css/news-item.css, static/css/news-item.css), and updated contents/structures/news.json and docs/index.html to expose the new item on the site. build.py: added render_news_pages() and copy_news_images(), integrated them into the main build flow, and fixed image-size lookup logic during WebP conversion. Also minor content fix to a member bio and added several layout/CSS tweaks for news and section links.
</commit_message>
<xml_diff>
--- a/contents/member-info.xlsx
+++ b/contents/member-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/Github/NTU-E3-Center.github.io/contents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79114A5-CC33-5441-972A-FC31918539D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCAA57C-0A87-2B46-90C0-BD26930F8B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -375,9 +375,6 @@
     <t>'25</t>
   </si>
   <si>
-    <t>Leo, also known by the nickname **DuoDuo(多多)**, completed his **undergraduate degree in Civil Engineering** at National Taiwan University (NTU) in 2025. He is currently a member of the **Computer-Aided Engineering (CAE)** division of NTU’s Civil Engineering department. His interests include playing volleyball, board games, and exploring new experiences. His research focuses on integrating **large language models (LLMs)** with **computer vision** to control autonomous vehicles, aiming to ensure safe driving, provide transparent explanations of model decisions, and optimize energy efficiency.</t>
-  </si>
-  <si>
     <t>/ Autonomous Vehicles 
 / Computer Vision</t>
   </si>
@@ -819,6 +816,9 @@
     <t>Year 1 Master's Student,
 Department of Chemical Engineering,
 National Taiwan University</t>
+  </si>
+  <si>
+    <t>Leo, also known by the nickname **DuoDuo** (多多), completed his **undergraduate degree in Civil Engineering** at National Taiwan University (NTU) in 2025. He is currently a member of the **Computer-Aided Engineering (CAE)** division of NTU’s Civil Engineering department. His interests include playing volleyball, board games, and exploring new experiences. His research focuses on integrating **large language models (LLMs)** with **computer vision** to control autonomous vehicles, aiming to ensure safe driving, provide transparent explanations of model decisions, and optimize energy efficiency.</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>2</v>
@@ -1278,7 +1278,7 @@
         <v>44</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H2" s="1" t="str">
         <f t="shared" ref="H2:H38" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(G2),"-","")," ",""))</f>
@@ -1333,7 +1333,7 @@
         <v>27</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H3" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1388,7 +1388,7 @@
         <v>38</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H4" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1490,13 +1490,13 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H6" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1543,7 +1543,7 @@
         <v>59</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H7" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1565,11 +1565,11 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Q7" s="1"/>
       <c r="R7" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -1616,7 +1616,7 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Q8" s="1" t="s">
         <v>69</v>
@@ -1645,7 +1645,7 @@
         <v>74</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H9" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1669,7 +1669,7 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>76</v>
@@ -1683,7 +1683,7 @@
         <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>79</v>
@@ -1692,13 +1692,13 @@
         <v>57</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H10" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>82</v>
@@ -1720,7 +1720,7 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -1745,7 +1745,7 @@
         <v>95</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H11" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1767,7 +1767,7 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
@@ -1792,7 +1792,7 @@
         <v>85</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H12" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1814,7 +1814,7 @@
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -1839,7 +1839,7 @@
         <v>81</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H13" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1861,7 +1861,7 @@
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
@@ -1910,7 +1910,7 @@
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q14" s="1" t="s">
         <v>92</v>
@@ -1933,23 +1933,23 @@
         <v>57</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="H15" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yifangchang</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>82</v>
@@ -1963,13 +1963,13 @@
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2016,13 +2016,13 @@
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>103</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2039,23 +2039,23 @@
         <v>87</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="H17" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yurankeng</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>82</v>
@@ -2069,13 +2069,13 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2092,13 +2092,13 @@
         <v>57</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H18" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>82</v>
@@ -2120,7 +2120,7 @@
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
@@ -2139,23 +2139,23 @@
         <v>57</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="G19" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H19" s="1" t="str">
         <f t="shared" si="0"/>
         <v>houchuanchen</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>82</v>
@@ -2169,13 +2169,13 @@
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="80" x14ac:dyDescent="0.2">
@@ -2192,13 +2192,13 @@
         <v>87</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="G20" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H20" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>82</v>
@@ -2220,7 +2220,7 @@
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
@@ -2230,22 +2230,22 @@
         <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="G21" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H21" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2253,13 +2253,13 @@
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>82</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M21" s="1" t="s">
         <v>67</v>
@@ -2267,7 +2267,7 @@
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
@@ -2277,22 +2277,22 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="G22" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H22" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2300,13 +2300,13 @@
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>82</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>67</v>
@@ -2314,7 +2314,7 @@
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
@@ -2324,22 +2324,22 @@
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="G23" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H23" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2347,13 +2347,13 @@
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>82</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>67</v>
@@ -2361,7 +2361,7 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
@@ -2371,22 +2371,22 @@
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H24" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2394,13 +2394,13 @@
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>82</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>67</v>
@@ -2408,7 +2408,7 @@
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
@@ -2418,35 +2418,35 @@
         <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="G25" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H25" s="1" t="str">
         <f t="shared" si="0"/>
         <v>chunhaohuang</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K25" s="1" t="s">
         <v>82</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M25" s="1" t="s">
         <v>67</v>
@@ -2454,7 +2454,7 @@
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
@@ -2464,32 +2464,32 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H26" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yugoimoto</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>52</v>
@@ -2510,35 +2510,35 @@
         <v>24</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="H27" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>chiayutsai</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="H27" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>chiayutsai</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="K27" s="1" t="s">
+      <c r="L27" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>31</v>
@@ -2554,35 +2554,35 @@
         <v>25</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="H28" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>tsunghengchang</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L28" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="H28" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>tsunghengchang</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>31</v>
@@ -2598,7 +2598,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>24</v>
@@ -2607,23 +2607,23 @@
         <v>57</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>167</v>
-      </c>
       <c r="G29" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H29" s="1" t="str">
         <f t="shared" si="0"/>
         <v>kaiyunlo</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L29" s="1" t="s">
         <v>30</v>
@@ -2642,7 +2642,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>24</v>
@@ -2654,20 +2654,20 @@
         <v>37</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H30" s="1" t="str">
         <f t="shared" si="0"/>
         <v>weihsuanchen</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L30" s="1" t="s">
         <v>30</v>
@@ -2686,7 +2686,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>24</v>
@@ -2695,23 +2695,23 @@
         <v>57</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>170</v>
-      </c>
       <c r="G31" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H31" s="1" t="str">
         <f t="shared" si="0"/>
         <v>yifanfeng</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L31" s="1" t="s">
         <v>30</v>
@@ -2730,7 +2730,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>36</v>
@@ -2739,13 +2739,13 @@
         <v>87</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="G32" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H32" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2753,10 +2753,10 @@
       </c>
       <c r="I32" s="1"/>
       <c r="J32" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>39</v>
@@ -2775,7 +2775,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>36</v>
@@ -2784,13 +2784,13 @@
         <v>57</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="G33" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H33" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2798,10 +2798,10 @@
       </c>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>39</v>
@@ -2820,7 +2820,7 @@
         <v>31</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>36</v>
@@ -2829,26 +2829,26 @@
         <v>57</v>
       </c>
       <c r="E34" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="H34" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>yuanhsichien</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="H34" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>yuanhsichien</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="J34" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>39</v>
@@ -2859,11 +2859,11 @@
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q34" s="1"/>
       <c r="R34" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
@@ -2871,7 +2871,7 @@
         <v>32</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>48</v>
@@ -2880,13 +2880,13 @@
         <v>87</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H35" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2894,10 +2894,10 @@
       </c>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>52</v>
@@ -2916,7 +2916,7 @@
         <v>33</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>48</v>
@@ -2925,13 +2925,13 @@
         <v>87</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>188</v>
-      </c>
       <c r="G36" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H36" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2939,10 +2939,10 @@
       </c>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>52</v>
@@ -2961,7 +2961,7 @@
         <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>48</v>
@@ -2970,13 +2970,13 @@
         <v>57</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="G37" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H37" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2984,10 +2984,10 @@
       </c>
       <c r="I37" s="1"/>
       <c r="J37" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L37" s="1" t="s">
         <v>52</v>
@@ -3006,7 +3006,7 @@
         <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>48</v>
@@ -3015,13 +3015,13 @@
         <v>57</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>199</v>
-      </c>
       <c r="G38" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H38" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3029,10 +3029,10 @@
       </c>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
content: consolidate director name link in about, add member interest entries
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contents/member-info.xlsx
+++ b/contents/member-info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/Github/NTU-E3-Center.github.io/contents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCAA57C-0A87-2B46-90C0-BD26930F8B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D02D851-FDCC-804D-AE7D-C59032AD2142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="246">
   <si>
     <t>WebID</t>
   </si>
@@ -819,6 +819,15 @@
   </si>
   <si>
     <t>Leo, also known by the nickname **DuoDuo** (多多), completed his **undergraduate degree in Civil Engineering** at National Taiwan University (NTU) in 2025. He is currently a member of the **Computer-Aided Engineering (CAE)** division of NTU’s Civil Engineering department. His interests include playing volleyball, board games, and exploring new experiences. His research focuses on integrating **large language models (LLMs)** with **computer vision** to control autonomous vehicles, aiming to ensure safe driving, provide transparent explanations of model decisions, and optimize energy efficiency.</t>
+  </si>
+  <si>
+    <t>/Energy System Optimization
+/Vehicle-to-Building (V2B) Strategy</t>
+  </si>
+  <si>
+    <t>/Smart Grid Modeling
+/Energy Management Systems
+/Low Carbon Logistics</t>
   </si>
 </sst>
 </file>
@@ -1473,7 +1482,9 @@
       <c r="P5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Q5" s="1"/>
+      <c r="Q5" s="1" t="s">
+        <v>244</v>
+      </c>
       <c r="R5" s="1" t="s">
         <v>53</v>
       </c>
@@ -1518,7 +1529,9 @@
       <c r="P6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" s="1"/>
+      <c r="Q6" s="1" t="s">
+        <v>245</v>
+      </c>
       <c r="R6" s="1" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
content+ux: promote contact to standalone subpage, update member content
</commit_message>
<xml_diff>
--- a/contents/member-info.xlsx
+++ b/contents/member-info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/NTU-E3-Center.github.io/contents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32519EFD-E392-D441-B682-16A23BC3E5DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02C2C1C-E0DF-DE42-96E9-DC2C07AA2991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="266">
   <si>
     <t>WebID</t>
   </si>
@@ -875,9 +875,6 @@
     <t>https://www.facebook.com/sean.shei/</t>
   </si>
   <si>
-    <t>www.linkedin.com/in/sean-shei-61409b293</t>
-  </si>
-  <si>
     <t>0009-0001-5290-5544</t>
   </si>
   <si>
@@ -885,6 +882,14 @@
   </si>
   <si>
     <t>https://scholar.google.com/citations?user=qG7wiMEAAAAJ</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/sean-shei-61409b293/</t>
+  </si>
+  <si>
+    <t>/Distributional Impacts of Climate and Energy Policy
+/Climate Policy and Global Inequality
+/Energy Transition and Electricity Market Reform</t>
   </si>
 </sst>
 </file>
@@ -1515,20 +1520,23 @@
       <c r="P4" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="Q4" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="R4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="T4" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="W4" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>261</v>
       </c>
       <c r="Y4" s="2" t="s">
         <v>260</v>

</xml_diff>

<commit_message>
content: update member info (xlsx + regenerated JSONs)
</commit_message>
<xml_diff>
--- a/contents/member-info.xlsx
+++ b/contents/member-info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/NTU-E3-Center.github.io/contents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02C2C1C-E0DF-DE42-96E9-DC2C07AA2991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6195BE-FE7B-FF47-888D-C4DC48EDC4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="29400" windowHeight="18480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="272">
   <si>
     <t>WebID</t>
   </si>
@@ -890,6 +890,24 @@
     <t>/Distributional Impacts of Climate and Energy Policy
 /Climate Policy and Global Inequality
 /Energy Transition and Electricity Market Reform</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=Djvdd44AAAAJ</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=JfG80RsAAAAJ</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=-hlSIJgAAAAJ</t>
+  </si>
+  <si>
+    <t>0009-0001-4608-919X</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/profile/Jian-Hern-Yeoh</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/jianhern/</t>
   </si>
 </sst>
 </file>
@@ -1598,6 +1616,18 @@
       <c r="R5" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="T5" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>271</v>
+      </c>
     </row>
     <row r="6" spans="1:25" ht="304" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1706,6 +1736,9 @@
       <c r="R7" s="1" t="s">
         <v>206</v>
       </c>
+      <c r="T7" s="2" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="8" spans="1:25" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1807,6 +1840,9 @@
       </c>
       <c r="R9" s="1" t="s">
         <v>75</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="112" x14ac:dyDescent="0.2">
@@ -3068,6 +3104,11 @@
     <hyperlink ref="U4" r:id="rId8" display="https://orcid.org/0009-0001-5290-5544" xr:uid="{A5D22604-2496-BE4F-B9DD-562C5B47E295}"/>
     <hyperlink ref="V4" r:id="rId9" xr:uid="{D172C527-C1C4-C047-A757-BC75CC7426F9}"/>
     <hyperlink ref="T4" r:id="rId10" xr:uid="{6F8425CF-B855-5A4A-B2B6-34D12B80B2AB}"/>
+    <hyperlink ref="T5" r:id="rId11" xr:uid="{4B38D0AD-2FC7-464D-9060-0D0FBCDDA9CB}"/>
+    <hyperlink ref="T7" r:id="rId12" xr:uid="{C7B4F0EB-6958-F54A-AF58-5BDA16E41654}"/>
+    <hyperlink ref="T9" r:id="rId13" xr:uid="{E2673CF1-94A5-2249-916F-2DCC53FC5CC1}"/>
+    <hyperlink ref="V5" r:id="rId14" xr:uid="{5AE67EF2-5E71-864C-90FE-CC4C98072E15}"/>
+    <hyperlink ref="W5" r:id="rId15" xr:uid="{C859D6CF-4C2E-2746-B2B4-BC6D99CC40FD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>